<commit_message>
Cost and claims histograms from the panel on one axis; Builty cost floor and ceiling in complete.do; elevations-by-state and summary-table updates
</commit_message>
<xml_diff>
--- a/output/tables/elevations_by_state.xlsx
+++ b/output/tables/elevations_by_state.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="93" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="96" uniqueCount="95">
   <si>
     <t>State</t>
   </si>
@@ -114,12 +114,12 @@
     <t>Nebraska</t>
   </si>
   <si>
+    <t>Montana</t>
+  </si>
+  <si>
     <t>Maine</t>
   </si>
   <si>
-    <t>Montana</t>
-  </si>
-  <si>
     <t>Tennessee</t>
   </si>
   <si>
@@ -132,12 +132,12 @@
     <t>Idaho</t>
   </si>
   <si>
+    <t>Arkansas</t>
+  </si>
+  <si>
     <t>Iowa</t>
   </si>
   <si>
-    <t>Arkansas</t>
-  </si>
-  <si>
     <t>New Hampshire</t>
   </si>
   <si>
@@ -243,12 +243,12 @@
     <t>NE</t>
   </si>
   <si>
+    <t>MT</t>
+  </si>
+  <si>
     <t>ME</t>
   </si>
   <si>
-    <t>MT</t>
-  </si>
-  <si>
     <t>TN</t>
   </si>
   <si>
@@ -261,12 +261,12 @@
     <t>ID</t>
   </si>
   <si>
+    <t>AR</t>
+  </si>
+  <si>
     <t>IA</t>
   </si>
   <si>
-    <t>AR</t>
-  </si>
-  <si>
     <t>NH</t>
   </si>
   <si>
@@ -289,6 +289,15 @@
   </si>
   <si>
     <t>Other HMA programs (properties)</t>
+  </si>
+  <si>
+    <t>NFIP elevations: flag flip or ICC payment (properties)</t>
+  </si>
+  <si>
+    <t>NFIP elevated flag flips 0 to 1 (properties)</t>
+  </si>
+  <si>
+    <t>NFIP ICC payment received (properties)</t>
   </si>
 </sst>
 </file>
@@ -334,7 +343,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -359,6 +368,15 @@
       <c r="G1" t="s">
         <v>91</v>
       </c>
+      <c r="H1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J1" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -382,6 +400,15 @@
       <c r="G2" s="1">
         <v>58</v>
       </c>
+      <c r="H2" s="1">
+        <v>1702</v>
+      </c>
+      <c r="I2" s="1">
+        <v>810</v>
+      </c>
+      <c r="J2" s="1">
+        <v>903</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -405,6 +432,15 @@
       <c r="G3" s="1">
         <v>5</v>
       </c>
+      <c r="H3" s="1">
+        <v>9192</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1131</v>
+      </c>
+      <c r="J3" s="1">
+        <v>8197</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
@@ -428,6 +464,15 @@
       <c r="G4" s="1">
         <v>17</v>
       </c>
+      <c r="H4" s="1">
+        <v>1448</v>
+      </c>
+      <c r="I4" s="1">
+        <v>649</v>
+      </c>
+      <c r="J4" s="1">
+        <v>815</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
@@ -451,6 +496,15 @@
       <c r="G5" s="1">
         <v>15</v>
       </c>
+      <c r="H5" s="1">
+        <v>1503</v>
+      </c>
+      <c r="I5" s="1">
+        <v>663</v>
+      </c>
+      <c r="J5" s="1">
+        <v>845</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -474,6 +528,15 @@
       <c r="G6" s="1">
         <v>15</v>
       </c>
+      <c r="H6" s="1">
+        <v>866</v>
+      </c>
+      <c r="I6" s="1">
+        <v>715</v>
+      </c>
+      <c r="J6" s="1">
+        <v>151</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
@@ -497,6 +560,15 @@
       <c r="G7" s="1">
         <v>16</v>
       </c>
+      <c r="H7" s="1">
+        <v>1676</v>
+      </c>
+      <c r="I7" s="1">
+        <v>779</v>
+      </c>
+      <c r="J7" s="1">
+        <v>900</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
@@ -520,6 +592,15 @@
       <c r="G8" s="1">
         <v>0</v>
       </c>
+      <c r="H8" s="1">
+        <v>2649</v>
+      </c>
+      <c r="I8" s="1">
+        <v>943</v>
+      </c>
+      <c r="J8" s="1">
+        <v>1775</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
@@ -543,6 +624,15 @@
       <c r="G9" s="1">
         <v>17</v>
       </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
@@ -566,6 +656,15 @@
       <c r="G10" s="1">
         <v>25</v>
       </c>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
@@ -589,6 +688,15 @@
       <c r="G11" s="1">
         <v>33</v>
       </c>
+      <c r="H11" s="1">
+        <v>208</v>
+      </c>
+      <c r="I11" s="1">
+        <v>191</v>
+      </c>
+      <c r="J11" s="1">
+        <v>18</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
@@ -612,6 +720,15 @@
       <c r="G12" s="1">
         <v>13</v>
       </c>
+      <c r="H12" s="1">
+        <v>465</v>
+      </c>
+      <c r="I12" s="1">
+        <v>162</v>
+      </c>
+      <c r="J12" s="1">
+        <v>309</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
@@ -635,6 +752,15 @@
       <c r="G13" s="1">
         <v>0</v>
       </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
@@ -658,6 +784,15 @@
       <c r="G14" s="1">
         <v>4</v>
       </c>
+      <c r="H14" s="1">
+        <v>313</v>
+      </c>
+      <c r="I14" s="1">
+        <v>283</v>
+      </c>
+      <c r="J14" s="1">
+        <v>30</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
@@ -681,6 +816,15 @@
       <c r="G15" s="1">
         <v>25</v>
       </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
@@ -704,6 +848,15 @@
       <c r="G16" s="1">
         <v>1</v>
       </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>0</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
@@ -727,6 +880,15 @@
       <c r="G17" s="1">
         <v>29</v>
       </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
@@ -750,6 +912,15 @@
       <c r="G18" s="1">
         <v>0</v>
       </c>
+      <c r="H18" s="1">
+        <v>561</v>
+      </c>
+      <c r="I18" s="1">
+        <v>198</v>
+      </c>
+      <c r="J18" s="1">
+        <v>365</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
@@ -773,6 +944,15 @@
       <c r="G19" s="1">
         <v>16</v>
       </c>
+      <c r="H19" s="1">
+        <v>435</v>
+      </c>
+      <c r="I19" s="1">
+        <v>311</v>
+      </c>
+      <c r="J19" s="1">
+        <v>125</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
@@ -796,6 +976,15 @@
       <c r="G20" s="1">
         <v>4</v>
       </c>
+      <c r="H20" s="1">
+        <v>625</v>
+      </c>
+      <c r="I20" s="1">
+        <v>501</v>
+      </c>
+      <c r="J20" s="1">
+        <v>126</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
@@ -819,6 +1008,15 @@
       <c r="G21" s="1">
         <v>0</v>
       </c>
+      <c r="H21" s="1">
+        <v>165</v>
+      </c>
+      <c r="I21" s="1">
+        <v>124</v>
+      </c>
+      <c r="J21" s="1">
+        <v>41</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
@@ -842,6 +1040,15 @@
       <c r="G22" s="1">
         <v>10</v>
       </c>
+      <c r="H22" s="1">
+        <v>93</v>
+      </c>
+      <c r="I22" s="1">
+        <v>85</v>
+      </c>
+      <c r="J22" s="1">
+        <v>8</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
@@ -865,6 +1072,15 @@
       <c r="G23" s="1">
         <v>0</v>
       </c>
+      <c r="H23" s="1">
+        <v>0</v>
+      </c>
+      <c r="I23" s="1">
+        <v>0</v>
+      </c>
+      <c r="J23" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
@@ -888,6 +1104,15 @@
       <c r="G24" s="1">
         <v>0</v>
       </c>
+      <c r="H24" s="1">
+        <v>262</v>
+      </c>
+      <c r="I24" s="1">
+        <v>92</v>
+      </c>
+      <c r="J24" s="1">
+        <v>170</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
@@ -911,6 +1136,15 @@
       <c r="G25" s="1">
         <v>13</v>
       </c>
+      <c r="H25" s="1">
+        <v>0</v>
+      </c>
+      <c r="I25" s="1">
+        <v>0</v>
+      </c>
+      <c r="J25" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
@@ -934,6 +1168,15 @@
       <c r="G26" s="1">
         <v>0</v>
       </c>
+      <c r="H26" s="1">
+        <v>93</v>
+      </c>
+      <c r="I26" s="1">
+        <v>72</v>
+      </c>
+      <c r="J26" s="1">
+        <v>21</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
@@ -957,6 +1200,15 @@
       <c r="G27" s="1">
         <v>0</v>
       </c>
+      <c r="H27" s="1">
+        <v>33</v>
+      </c>
+      <c r="I27" s="1">
+        <v>9</v>
+      </c>
+      <c r="J27" s="1">
+        <v>24</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
@@ -980,6 +1232,15 @@
       <c r="G28" s="1">
         <v>0</v>
       </c>
+      <c r="H28" s="1">
+        <v>0</v>
+      </c>
+      <c r="I28" s="1">
+        <v>0</v>
+      </c>
+      <c r="J28" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
@@ -1003,6 +1264,15 @@
       <c r="G29" s="1">
         <v>0</v>
       </c>
+      <c r="H29" s="1">
+        <v>0</v>
+      </c>
+      <c r="I29" s="1">
+        <v>0</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
@@ -1026,6 +1296,15 @@
       <c r="G30" s="1">
         <v>0</v>
       </c>
+      <c r="H30" s="1">
+        <v>0</v>
+      </c>
+      <c r="I30" s="1">
+        <v>0</v>
+      </c>
+      <c r="J30" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
@@ -1049,6 +1328,15 @@
       <c r="G31" s="1">
         <v>10</v>
       </c>
+      <c r="H31" s="1">
+        <v>0</v>
+      </c>
+      <c r="I31" s="1">
+        <v>0</v>
+      </c>
+      <c r="J31" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
@@ -1072,6 +1360,15 @@
       <c r="G32" s="1">
         <v>0</v>
       </c>
+      <c r="H32" s="1">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1">
+        <v>0</v>
+      </c>
+      <c r="J32" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
@@ -1095,6 +1392,15 @@
       <c r="G33" s="1">
         <v>0</v>
       </c>
+      <c r="H33" s="1">
+        <v>0</v>
+      </c>
+      <c r="I33" s="1">
+        <v>0</v>
+      </c>
+      <c r="J33" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
@@ -1110,12 +1416,21 @@
         <v>8</v>
       </c>
       <c r="E34" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F34" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G34" s="1">
+        <v>0</v>
+      </c>
+      <c r="H34" s="1">
+        <v>0</v>
+      </c>
+      <c r="I34" s="1">
+        <v>0</v>
+      </c>
+      <c r="J34" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1133,13 +1448,22 @@
         <v>8</v>
       </c>
       <c r="E35" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F35" s="1">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G35" s="1">
         <v>0</v>
+      </c>
+      <c r="H35" s="1">
+        <v>31</v>
+      </c>
+      <c r="I35" s="1">
+        <v>28</v>
+      </c>
+      <c r="J35" s="1">
+        <v>3</v>
       </c>
     </row>
     <row r="36">
@@ -1164,6 +1488,15 @@
       <c r="G36" s="1">
         <v>0</v>
       </c>
+      <c r="H36" s="1">
+        <v>0</v>
+      </c>
+      <c r="I36" s="1">
+        <v>0</v>
+      </c>
+      <c r="J36" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
@@ -1187,6 +1520,15 @@
       <c r="G37" s="1">
         <v>7</v>
       </c>
+      <c r="H37" s="1">
+        <v>0</v>
+      </c>
+      <c r="I37" s="1">
+        <v>0</v>
+      </c>
+      <c r="J37" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
@@ -1210,6 +1552,15 @@
       <c r="G38" s="1">
         <v>0</v>
       </c>
+      <c r="H38" s="1">
+        <v>0</v>
+      </c>
+      <c r="I38" s="1">
+        <v>0</v>
+      </c>
+      <c r="J38" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
@@ -1233,6 +1584,15 @@
       <c r="G39" s="1">
         <v>0</v>
       </c>
+      <c r="H39" s="1">
+        <v>0</v>
+      </c>
+      <c r="I39" s="1">
+        <v>0</v>
+      </c>
+      <c r="J39" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
@@ -1256,6 +1616,15 @@
       <c r="G40" s="1">
         <v>0</v>
       </c>
+      <c r="H40" s="1">
+        <v>0</v>
+      </c>
+      <c r="I40" s="1">
+        <v>0</v>
+      </c>
+      <c r="J40" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
@@ -1279,6 +1648,15 @@
       <c r="G41" s="1">
         <v>0</v>
       </c>
+      <c r="H41" s="1">
+        <v>0</v>
+      </c>
+      <c r="I41" s="1">
+        <v>0</v>
+      </c>
+      <c r="J41" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
@@ -1302,6 +1680,15 @@
       <c r="G42" s="1">
         <v>1</v>
       </c>
+      <c r="H42" s="1">
+        <v>35</v>
+      </c>
+      <c r="I42" s="1">
+        <v>31</v>
+      </c>
+      <c r="J42" s="1">
+        <v>4</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
@@ -1325,6 +1712,15 @@
       <c r="G43" s="1">
         <v>0</v>
       </c>
+      <c r="H43" s="1">
+        <v>0</v>
+      </c>
+      <c r="I43" s="1">
+        <v>0</v>
+      </c>
+      <c r="J43" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
@@ -1348,6 +1744,15 @@
       <c r="G44" s="1">
         <v>0</v>
       </c>
+      <c r="H44" s="1">
+        <v>0</v>
+      </c>
+      <c r="I44" s="1">
+        <v>0</v>
+      </c>
+      <c r="J44" s="1">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>